<commit_message>
Refactor UI and Database Integration
- Updated the UI to support database connections and dataset loading.
- Enhanced the `ApplyRules` function to handle datasets more effectively.
- Introduced database export functionality with `ExportToDB` for SQLite and other drivers.
- Added tests for database operations and dataset loading.
- Improved dataset handling in the UI, allowing for better user interaction and data manipulation.
- Added configuration for transformers in the UI to support various data types and formats.
- Updated the test dataset to include a comprehensive configuration for supermarket sales.
</commit_message>
<xml_diff>
--- a/test/Supermarket-Sales-Sample-Data.xlsx
+++ b/test/Supermarket-Sales-Sample-Data.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="SuperMarket Sales" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="SuperMarket Sales" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="daily" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="130">
   <si>
     <t xml:space="preserve">Order No</t>
   </si>
@@ -404,6 +405,12 @@
   </si>
   <si>
     <t xml:space="preserve">1070</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vente</t>
   </si>
 </sst>
 </file>
@@ -516,28 +523,32 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -613,13 +624,119 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="FFFFFF"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18A303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369A3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A33E03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8E03A3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="C99C00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="C9211E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000EE"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551A8B"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G73"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.87890625" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.66"/>
@@ -628,49 +745,49 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="19.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="17.33"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1021" min="7" style="1" width="8.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1022" style="0" width="12.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1022" style="2" width="12.83"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="5" t="n">
         <v>45292</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="5" t="n">
         <v>45294</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="4" t="n">
         <v>49.99</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F2" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G2" s="1" t="n">
@@ -679,22 +796,22 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="5" t="n">
         <v>45292</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="5" t="n">
         <v>45295</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" s="4" t="n">
         <v>29.99</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="F3" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G3" s="1" t="n">
@@ -703,22 +820,22 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="5" t="n">
         <v>45293</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="5" t="n">
         <v>45298</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="4" t="n">
         <v>99.99</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F4" s="4" t="n">
         <v>3</v>
       </c>
       <c r="G4" s="1" t="n">
@@ -727,22 +844,22 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="5" t="n">
         <v>45293</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="5" t="n">
         <v>45294</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="4" t="n">
         <v>19.99</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="F5" s="4" t="n">
         <v>4</v>
       </c>
       <c r="G5" s="1" t="n">
@@ -751,22 +868,22 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="5" t="n">
         <v>45294</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="5" t="n">
         <v>45299</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="E6" s="4" t="n">
         <v>149.99</v>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="F6" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G6" s="1" t="n">
@@ -775,22 +892,22 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="5" t="n">
         <v>45294</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="5" t="n">
         <v>45297</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="E7" s="4" t="n">
         <v>79.99</v>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="F7" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G7" s="1" t="n">
@@ -799,22 +916,22 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="5" t="n">
         <v>45295</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="5" t="n">
         <v>45297</v>
       </c>
-      <c r="E8" s="3" t="n">
+      <c r="E8" s="4" t="n">
         <v>39.99</v>
       </c>
-      <c r="F8" s="3" t="n">
+      <c r="F8" s="4" t="n">
         <v>3</v>
       </c>
       <c r="G8" s="1" t="n">
@@ -823,22 +940,22 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="5" t="n">
         <v>45295</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="5" t="n">
         <v>45300</v>
       </c>
-      <c r="E9" s="3" t="n">
+      <c r="E9" s="4" t="n">
         <v>69.99</v>
       </c>
-      <c r="F9" s="3" t="n">
+      <c r="F9" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G9" s="1" t="n">
@@ -847,22 +964,22 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B10" s="5" t="n">
         <v>45296</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="5" t="n">
         <v>45297</v>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="E10" s="4" t="n">
         <v>89.99</v>
       </c>
-      <c r="F10" s="3" t="n">
+      <c r="F10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="1" t="n">
@@ -871,22 +988,22 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B11" s="5" t="n">
         <v>45296</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="5" t="n">
         <v>45299</v>
       </c>
-      <c r="E11" s="3" t="n">
+      <c r="E11" s="4" t="n">
         <v>199.99</v>
       </c>
-      <c r="F11" s="3" t="n">
+      <c r="F11" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G11" s="1" t="n">
@@ -895,22 +1012,22 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="4" t="n">
+      <c r="B12" s="5" t="n">
         <v>45297</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" s="5" t="n">
         <v>45298</v>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="E12" s="4" t="n">
         <v>29.99</v>
       </c>
-      <c r="F12" s="3" t="n">
+      <c r="F12" s="4" t="n">
         <v>5</v>
       </c>
       <c r="G12" s="1" t="n">
@@ -919,22 +1036,22 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B13" s="5" t="n">
         <v>45297</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="5" t="n">
         <v>45299</v>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="E13" s="4" t="n">
         <v>79.99</v>
       </c>
-      <c r="F13" s="3" t="n">
+      <c r="F13" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G13" s="1" t="n">
@@ -943,22 +1060,22 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="5" t="n">
         <v>45298</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D14" s="5" t="n">
         <v>45300</v>
       </c>
-      <c r="E14" s="3" t="n">
+      <c r="E14" s="4" t="n">
         <v>49.99</v>
       </c>
-      <c r="F14" s="3" t="n">
+      <c r="F14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="G14" s="1" t="n">
@@ -967,22 +1084,22 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B15" s="4" t="n">
+      <c r="B15" s="5" t="n">
         <v>45298</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="D15" s="5" t="n">
         <v>45303</v>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="E15" s="4" t="n">
         <v>129.99</v>
       </c>
-      <c r="F15" s="3" t="n">
+      <c r="F15" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G15" s="1" t="n">
@@ -991,22 +1108,22 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="4" t="n">
+      <c r="B16" s="5" t="n">
         <v>45299</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="D16" s="5" t="n">
         <v>45304</v>
       </c>
-      <c r="E16" s="3" t="n">
+      <c r="E16" s="4" t="n">
         <v>19.99</v>
       </c>
-      <c r="F16" s="3" t="n">
+      <c r="F16" s="4" t="n">
         <v>4</v>
       </c>
       <c r="G16" s="1" t="n">
@@ -1015,22 +1132,22 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="4" t="n">
+      <c r="B17" s="5" t="n">
         <v>45299</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="D17" s="5" t="n">
         <v>45303</v>
       </c>
-      <c r="E17" s="3" t="n">
+      <c r="E17" s="4" t="n">
         <v>149.99</v>
       </c>
-      <c r="F17" s="3" t="n">
+      <c r="F17" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G17" s="1" t="n">
@@ -1039,22 +1156,22 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="4" t="n">
+      <c r="B18" s="5" t="n">
         <v>45300</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="D18" s="5" t="n">
         <v>45305</v>
       </c>
-      <c r="E18" s="3" t="n">
+      <c r="E18" s="4" t="n">
         <v>69.99</v>
       </c>
-      <c r="F18" s="3" t="n">
+      <c r="F18" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G18" s="1" t="n">
@@ -1063,22 +1180,22 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B19" s="4" t="n">
+      <c r="B19" s="5" t="n">
         <v>45300</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D19" s="4" t="n">
+      <c r="D19" s="5" t="n">
         <v>45303</v>
       </c>
-      <c r="E19" s="3" t="n">
+      <c r="E19" s="4" t="n">
         <v>39.99</v>
       </c>
-      <c r="F19" s="3" t="n">
+      <c r="F19" s="4" t="n">
         <v>3</v>
       </c>
       <c r="G19" s="1" t="n">
@@ -1087,22 +1204,22 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B20" s="4" t="n">
+      <c r="B20" s="5" t="n">
         <v>45301</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="D20" s="4" t="n">
+      <c r="D20" s="5" t="n">
         <v>45302</v>
       </c>
-      <c r="E20" s="3" t="n">
+      <c r="E20" s="4" t="n">
         <v>199.99</v>
       </c>
-      <c r="F20" s="3" t="n">
+      <c r="F20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G20" s="1" t="n">
@@ -1111,22 +1228,22 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="4" t="n">
+      <c r="B21" s="5" t="n">
         <v>45301</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D21" s="4" t="n">
+      <c r="D21" s="5" t="n">
         <v>45305</v>
       </c>
-      <c r="E21" s="3" t="n">
+      <c r="E21" s="4" t="n">
         <v>29.99</v>
       </c>
-      <c r="F21" s="3" t="n">
+      <c r="F21" s="4" t="n">
         <v>5</v>
       </c>
       <c r="G21" s="1" t="n">
@@ -1135,22 +1252,22 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="4" t="n">
+      <c r="B22" s="5" t="n">
         <v>45302</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D22" s="4" t="n">
+      <c r="D22" s="5" t="n">
         <v>45305</v>
       </c>
-      <c r="E22" s="3" t="n">
+      <c r="E22" s="4" t="n">
         <v>79.99</v>
       </c>
-      <c r="F22" s="3" t="n">
+      <c r="F22" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G22" s="1" t="n">
@@ -1159,22 +1276,22 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B23" s="4" t="n">
+      <c r="B23" s="5" t="n">
         <v>45302</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="D23" s="4" t="n">
+      <c r="D23" s="5" t="n">
         <v>45306</v>
       </c>
-      <c r="E23" s="3" t="n">
+      <c r="E23" s="4" t="n">
         <v>49.99</v>
       </c>
-      <c r="F23" s="3" t="n">
+      <c r="F23" s="4" t="n">
         <v>3</v>
       </c>
       <c r="G23" s="1" t="n">
@@ -1183,22 +1300,22 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B24" s="4" t="n">
+      <c r="B24" s="5" t="n">
         <v>45303</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D24" s="4" t="n">
+      <c r="D24" s="5" t="n">
         <v>45308</v>
       </c>
-      <c r="E24" s="3" t="n">
+      <c r="E24" s="4" t="n">
         <v>129.99</v>
       </c>
-      <c r="F24" s="3" t="n">
+      <c r="F24" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G24" s="1" t="n">
@@ -1207,22 +1324,22 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B25" s="4" t="n">
+      <c r="B25" s="5" t="n">
         <v>45303</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D25" s="4" t="n">
+      <c r="D25" s="5" t="n">
         <v>45308</v>
       </c>
-      <c r="E25" s="3" t="n">
+      <c r="E25" s="4" t="n">
         <v>19.99</v>
       </c>
-      <c r="F25" s="3" t="n">
+      <c r="F25" s="4" t="n">
         <v>4</v>
       </c>
       <c r="G25" s="1" t="n">
@@ -1231,22 +1348,22 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B26" s="4" t="n">
+      <c r="B26" s="5" t="n">
         <v>45304</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D26" s="4" t="n">
+      <c r="D26" s="5" t="n">
         <v>45308</v>
       </c>
-      <c r="E26" s="3" t="n">
+      <c r="E26" s="4" t="n">
         <v>149.99</v>
       </c>
-      <c r="F26" s="3" t="n">
+      <c r="F26" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G26" s="1" t="n">
@@ -1255,22 +1372,22 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
+      <c r="A27" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B27" s="4" t="n">
+      <c r="B27" s="5" t="n">
         <v>45304</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D27" s="4" t="n">
+      <c r="D27" s="5" t="n">
         <v>45305</v>
       </c>
-      <c r="E27" s="3" t="n">
+      <c r="E27" s="4" t="n">
         <v>69.99</v>
       </c>
-      <c r="F27" s="3" t="n">
+      <c r="F27" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G27" s="1" t="n">
@@ -1279,22 +1396,22 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B28" s="4" t="n">
+      <c r="B28" s="5" t="n">
         <v>45305</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D28" s="4" t="n">
+      <c r="D28" s="5" t="n">
         <v>45309</v>
       </c>
-      <c r="E28" s="3" t="n">
+      <c r="E28" s="4" t="n">
         <v>39.99</v>
       </c>
-      <c r="F28" s="3" t="n">
+      <c r="F28" s="4" t="n">
         <v>3</v>
       </c>
       <c r="G28" s="1" t="n">
@@ -1303,22 +1420,22 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
+      <c r="A29" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="4" t="n">
+      <c r="B29" s="5" t="n">
         <v>45305</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D29" s="4" t="n">
+      <c r="D29" s="5" t="n">
         <v>45310</v>
       </c>
-      <c r="E29" s="3" t="n">
+      <c r="E29" s="4" t="n">
         <v>199.99</v>
       </c>
-      <c r="F29" s="3" t="n">
+      <c r="F29" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G29" s="1" t="n">
@@ -1327,22 +1444,22 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
+      <c r="A30" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="4" t="n">
+      <c r="B30" s="5" t="n">
         <v>45306</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D30" s="4" t="n">
+      <c r="D30" s="5" t="n">
         <v>45310</v>
       </c>
-      <c r="E30" s="3" t="n">
+      <c r="E30" s="4" t="n">
         <v>29.99</v>
       </c>
-      <c r="F30" s="3" t="n">
+      <c r="F30" s="4" t="n">
         <v>5</v>
       </c>
       <c r="G30" s="1" t="n">
@@ -1351,22 +1468,22 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
+      <c r="A31" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B31" s="4" t="n">
+      <c r="B31" s="5" t="n">
         <v>45306</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C31" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D31" s="4" t="n">
+      <c r="D31" s="5" t="n">
         <v>45310</v>
       </c>
-      <c r="E31" s="3" t="n">
+      <c r="E31" s="4" t="n">
         <v>79.99</v>
       </c>
-      <c r="F31" s="3" t="n">
+      <c r="F31" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G31" s="1" t="n">
@@ -1375,22 +1492,22 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
+      <c r="A32" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B32" s="4" t="n">
+      <c r="B32" s="5" t="n">
         <v>45307</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="D32" s="4" t="n">
+      <c r="D32" s="5" t="n">
         <v>45310</v>
       </c>
-      <c r="E32" s="3" t="n">
+      <c r="E32" s="4" t="n">
         <v>49.99</v>
       </c>
-      <c r="F32" s="3" t="n">
+      <c r="F32" s="4" t="n">
         <v>3</v>
       </c>
       <c r="G32" s="1" t="n">
@@ -1399,22 +1516,22 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
+      <c r="A33" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B33" s="4" t="n">
+      <c r="B33" s="5" t="n">
         <v>45307</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C33" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="D33" s="4" t="n">
+      <c r="D33" s="5" t="n">
         <v>45308</v>
       </c>
-      <c r="E33" s="3" t="n">
+      <c r="E33" s="4" t="n">
         <v>129.99</v>
       </c>
-      <c r="F33" s="3" t="n">
+      <c r="F33" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G33" s="1" t="n">
@@ -1423,22 +1540,22 @@
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B34" s="4" t="n">
+      <c r="B34" s="5" t="n">
         <v>45308</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D34" s="4" t="n">
+      <c r="D34" s="5" t="n">
         <v>45310</v>
       </c>
-      <c r="E34" s="3" t="n">
+      <c r="E34" s="4" t="n">
         <v>19.99</v>
       </c>
-      <c r="F34" s="3" t="n">
+      <c r="F34" s="4" t="n">
         <v>4</v>
       </c>
       <c r="G34" s="1" t="n">
@@ -1447,22 +1564,22 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
+      <c r="A35" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B35" s="4" t="n">
+      <c r="B35" s="5" t="n">
         <v>45308</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="D35" s="4" t="n">
+      <c r="D35" s="5" t="n">
         <v>45310</v>
       </c>
-      <c r="E35" s="3" t="n">
+      <c r="E35" s="4" t="n">
         <v>149.99</v>
       </c>
-      <c r="F35" s="3" t="n">
+      <c r="F35" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G35" s="1" t="n">
@@ -1471,22 +1588,22 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3" t="s">
+      <c r="A36" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B36" s="4" t="n">
+      <c r="B36" s="5" t="n">
         <v>45309</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="C36" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="D36" s="4" t="n">
+      <c r="D36" s="5" t="n">
         <v>45314</v>
       </c>
-      <c r="E36" s="3" t="n">
+      <c r="E36" s="4" t="n">
         <v>69.99</v>
       </c>
-      <c r="F36" s="3" t="n">
+      <c r="F36" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G36" s="1" t="n">
@@ -1495,22 +1612,22 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="3" t="s">
+      <c r="A37" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B37" s="4" t="n">
+      <c r="B37" s="5" t="n">
         <v>45309</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="C37" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="D37" s="4" t="n">
+      <c r="D37" s="5" t="n">
         <v>45310</v>
       </c>
-      <c r="E37" s="3" t="n">
+      <c r="E37" s="4" t="n">
         <v>39.99</v>
       </c>
-      <c r="F37" s="3" t="n">
+      <c r="F37" s="4" t="n">
         <v>3</v>
       </c>
       <c r="G37" s="1" t="n">
@@ -1519,22 +1636,22 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="3" t="s">
+      <c r="A38" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B38" s="4" t="n">
+      <c r="B38" s="5" t="n">
         <v>45310</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="C38" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D38" s="4" t="n">
+      <c r="D38" s="5" t="n">
         <v>45311</v>
       </c>
-      <c r="E38" s="3" t="n">
+      <c r="E38" s="4" t="n">
         <v>199.99</v>
       </c>
-      <c r="F38" s="3" t="n">
+      <c r="F38" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G38" s="1" t="n">
@@ -1543,22 +1660,22 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3" t="s">
+      <c r="A39" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B39" s="4" t="n">
+      <c r="B39" s="5" t="n">
         <v>45310</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C39" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="D39" s="4" t="n">
+      <c r="D39" s="5" t="n">
         <v>45313</v>
       </c>
-      <c r="E39" s="3" t="n">
+      <c r="E39" s="4" t="n">
         <v>29.99</v>
       </c>
-      <c r="F39" s="3" t="n">
+      <c r="F39" s="4" t="n">
         <v>5</v>
       </c>
       <c r="G39" s="1" t="n">
@@ -1567,22 +1684,22 @@
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="s">
+      <c r="A40" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B40" s="4" t="n">
+      <c r="B40" s="5" t="n">
         <v>45311</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="C40" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D40" s="4" t="n">
+      <c r="D40" s="5" t="n">
         <v>45315</v>
       </c>
-      <c r="E40" s="3" t="n">
+      <c r="E40" s="4" t="n">
         <v>79.99</v>
       </c>
-      <c r="F40" s="3" t="n">
+      <c r="F40" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G40" s="1" t="n">
@@ -1591,22 +1708,22 @@
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="3" t="s">
+      <c r="A41" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="B41" s="4" t="n">
+      <c r="B41" s="5" t="n">
         <v>45311</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="C41" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D41" s="4" t="n">
+      <c r="D41" s="5" t="n">
         <v>45312</v>
       </c>
-      <c r="E41" s="3" t="n">
+      <c r="E41" s="4" t="n">
         <v>49.99</v>
       </c>
-      <c r="F41" s="3" t="n">
+      <c r="F41" s="4" t="n">
         <v>3</v>
       </c>
       <c r="G41" s="1" t="n">
@@ -1615,22 +1732,22 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3" t="s">
+      <c r="A42" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B42" s="4" t="n">
+      <c r="B42" s="5" t="n">
         <v>45312</v>
       </c>
-      <c r="C42" s="3" t="s">
+      <c r="C42" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D42" s="4" t="n">
+      <c r="D42" s="5" t="n">
         <v>45317</v>
       </c>
-      <c r="E42" s="3" t="n">
+      <c r="E42" s="4" t="n">
         <v>129.99</v>
       </c>
-      <c r="F42" s="3" t="n">
+      <c r="F42" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G42" s="1" t="n">
@@ -1639,22 +1756,22 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3" t="s">
+      <c r="A43" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B43" s="4" t="n">
+      <c r="B43" s="5" t="n">
         <v>45312</v>
       </c>
-      <c r="C43" s="3" t="s">
+      <c r="C43" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D43" s="4" t="n">
+      <c r="D43" s="5" t="n">
         <v>45314</v>
       </c>
-      <c r="E43" s="3" t="n">
+      <c r="E43" s="4" t="n">
         <v>19.99</v>
       </c>
-      <c r="F43" s="3" t="n">
+      <c r="F43" s="4" t="n">
         <v>4</v>
       </c>
       <c r="G43" s="1" t="n">
@@ -1663,22 +1780,22 @@
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="3" t="s">
+      <c r="A44" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B44" s="4" t="n">
+      <c r="B44" s="5" t="n">
         <v>45313</v>
       </c>
-      <c r="C44" s="3" t="s">
+      <c r="C44" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D44" s="4" t="n">
+      <c r="D44" s="5" t="n">
         <v>45316</v>
       </c>
-      <c r="E44" s="3" t="n">
+      <c r="E44" s="4" t="n">
         <v>149.99</v>
       </c>
-      <c r="F44" s="3" t="n">
+      <c r="F44" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G44" s="1" t="n">
@@ -1687,22 +1804,22 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="3" t="s">
+      <c r="A45" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B45" s="4" t="n">
+      <c r="B45" s="5" t="n">
         <v>45313</v>
       </c>
-      <c r="C45" s="3" t="s">
+      <c r="C45" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D45" s="4" t="n">
+      <c r="D45" s="5" t="n">
         <v>45316</v>
       </c>
-      <c r="E45" s="3" t="n">
+      <c r="E45" s="4" t="n">
         <v>69.99</v>
       </c>
-      <c r="F45" s="3" t="n">
+      <c r="F45" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G45" s="1" t="n">
@@ -1711,22 +1828,22 @@
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3" t="s">
+      <c r="A46" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B46" s="4" t="n">
+      <c r="B46" s="5" t="n">
         <v>45314</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C46" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="D46" s="4" t="n">
+      <c r="D46" s="5" t="n">
         <v>45318</v>
       </c>
-      <c r="E46" s="3" t="n">
+      <c r="E46" s="4" t="n">
         <v>39.99</v>
       </c>
-      <c r="F46" s="3" t="n">
+      <c r="F46" s="4" t="n">
         <v>3</v>
       </c>
       <c r="G46" s="1" t="n">
@@ -1735,22 +1852,22 @@
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3" t="s">
+      <c r="A47" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B47" s="4" t="n">
+      <c r="B47" s="5" t="n">
         <v>45314</v>
       </c>
-      <c r="C47" s="3" t="s">
+      <c r="C47" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D47" s="4" t="n">
+      <c r="D47" s="5" t="n">
         <v>45317</v>
       </c>
-      <c r="E47" s="3" t="n">
+      <c r="E47" s="4" t="n">
         <v>199.99</v>
       </c>
-      <c r="F47" s="3" t="n">
+      <c r="F47" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G47" s="1" t="n">
@@ -1759,22 +1876,22 @@
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="3" t="s">
+      <c r="A48" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B48" s="4" t="n">
+      <c r="B48" s="5" t="n">
         <v>45315</v>
       </c>
-      <c r="C48" s="3" t="s">
+      <c r="C48" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="D48" s="4" t="n">
+      <c r="D48" s="5" t="n">
         <v>45316</v>
       </c>
-      <c r="E48" s="3" t="n">
+      <c r="E48" s="4" t="n">
         <v>29.99</v>
       </c>
-      <c r="F48" s="3" t="n">
+      <c r="F48" s="4" t="n">
         <v>5</v>
       </c>
       <c r="G48" s="1" t="n">
@@ -1783,22 +1900,22 @@
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3" t="s">
+      <c r="A49" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="B49" s="4" t="n">
+      <c r="B49" s="5" t="n">
         <v>45315</v>
       </c>
-      <c r="C49" s="3" t="s">
+      <c r="C49" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D49" s="4" t="n">
+      <c r="D49" s="5" t="n">
         <v>45317</v>
       </c>
-      <c r="E49" s="3" t="n">
+      <c r="E49" s="4" t="n">
         <v>79.99</v>
       </c>
-      <c r="F49" s="3" t="n">
+      <c r="F49" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G49" s="1" t="n">
@@ -1807,22 +1924,22 @@
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="3" t="s">
+      <c r="A50" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="B50" s="4" t="n">
+      <c r="B50" s="5" t="n">
         <v>45316</v>
       </c>
-      <c r="C50" s="3" t="s">
+      <c r="C50" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="D50" s="4" t="n">
+      <c r="D50" s="5" t="n">
         <v>45321</v>
       </c>
-      <c r="E50" s="3" t="n">
+      <c r="E50" s="4" t="n">
         <v>49.99</v>
       </c>
-      <c r="F50" s="3" t="n">
+      <c r="F50" s="4" t="n">
         <v>3</v>
       </c>
       <c r="G50" s="1" t="n">
@@ -1831,22 +1948,22 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3" t="s">
+      <c r="A51" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="B51" s="4" t="n">
+      <c r="B51" s="5" t="n">
         <v>45316</v>
       </c>
-      <c r="C51" s="3" t="s">
+      <c r="C51" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="D51" s="4" t="n">
+      <c r="D51" s="5" t="n">
         <v>45318</v>
       </c>
-      <c r="E51" s="3" t="n">
+      <c r="E51" s="4" t="n">
         <v>129.99</v>
       </c>
-      <c r="F51" s="3" t="n">
+      <c r="F51" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G51" s="1" t="n">
@@ -1855,22 +1972,22 @@
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="3" t="s">
+      <c r="A52" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B52" s="4" t="n">
+      <c r="B52" s="5" t="n">
         <v>45317</v>
       </c>
-      <c r="C52" s="3" t="s">
+      <c r="C52" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="D52" s="4" t="n">
+      <c r="D52" s="5" t="n">
         <v>45320</v>
       </c>
-      <c r="E52" s="3" t="n">
+      <c r="E52" s="4" t="n">
         <v>19.99</v>
       </c>
-      <c r="F52" s="3" t="n">
+      <c r="F52" s="4" t="n">
         <v>4</v>
       </c>
       <c r="G52" s="1" t="n">
@@ -1879,22 +1996,22 @@
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3" t="s">
+      <c r="A53" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="B53" s="4" t="n">
+      <c r="B53" s="5" t="n">
         <v>45317</v>
       </c>
-      <c r="C53" s="3" t="s">
+      <c r="C53" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D53" s="4" t="n">
+      <c r="D53" s="5" t="n">
         <v>45319</v>
       </c>
-      <c r="E53" s="3" t="n">
+      <c r="E53" s="4" t="n">
         <v>149.99</v>
       </c>
-      <c r="F53" s="3" t="n">
+      <c r="F53" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G53" s="1" t="n">
@@ -1903,22 +2020,22 @@
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="3" t="s">
+      <c r="A54" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="B54" s="4" t="n">
+      <c r="B54" s="5" t="n">
         <v>45318</v>
       </c>
-      <c r="C54" s="3" t="s">
+      <c r="C54" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D54" s="4" t="n">
+      <c r="D54" s="5" t="n">
         <v>45322</v>
       </c>
-      <c r="E54" s="3" t="n">
+      <c r="E54" s="4" t="n">
         <v>69.99</v>
       </c>
-      <c r="F54" s="3" t="n">
+      <c r="F54" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G54" s="1" t="n">
@@ -1927,22 +2044,22 @@
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="3" t="s">
+      <c r="A55" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="B55" s="4" t="n">
+      <c r="B55" s="5" t="n">
         <v>45318</v>
       </c>
-      <c r="C55" s="3" t="s">
+      <c r="C55" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="D55" s="4" t="n">
+      <c r="D55" s="5" t="n">
         <v>45322</v>
       </c>
-      <c r="E55" s="3" t="n">
+      <c r="E55" s="4" t="n">
         <v>39.99</v>
       </c>
-      <c r="F55" s="3" t="n">
+      <c r="F55" s="4" t="n">
         <v>3</v>
       </c>
       <c r="G55" s="1" t="n">
@@ -1951,22 +2068,22 @@
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="3" t="s">
+      <c r="A56" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="B56" s="4" t="n">
+      <c r="B56" s="5" t="n">
         <v>45319</v>
       </c>
-      <c r="C56" s="3" t="s">
+      <c r="C56" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="D56" s="4" t="n">
+      <c r="D56" s="5" t="n">
         <v>45320</v>
       </c>
-      <c r="E56" s="3" t="n">
+      <c r="E56" s="4" t="n">
         <v>199.99</v>
       </c>
-      <c r="F56" s="3" t="n">
+      <c r="F56" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G56" s="1" t="n">
@@ -1975,22 +2092,22 @@
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="3" t="s">
+      <c r="A57" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="B57" s="4" t="n">
+      <c r="B57" s="5" t="n">
         <v>45319</v>
       </c>
-      <c r="C57" s="3" t="s">
+      <c r="C57" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="D57" s="4" t="n">
+      <c r="D57" s="5" t="n">
         <v>45320</v>
       </c>
-      <c r="E57" s="3" t="n">
+      <c r="E57" s="4" t="n">
         <v>29.99</v>
       </c>
-      <c r="F57" s="3" t="n">
+      <c r="F57" s="4" t="n">
         <v>5</v>
       </c>
       <c r="G57" s="1" t="n">
@@ -1999,22 +2116,22 @@
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="3" t="s">
+      <c r="A58" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="B58" s="4" t="n">
+      <c r="B58" s="5" t="n">
         <v>45320</v>
       </c>
-      <c r="C58" s="3" t="s">
+      <c r="C58" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="D58" s="4" t="n">
+      <c r="D58" s="5" t="n">
         <v>45321</v>
       </c>
-      <c r="E58" s="3" t="n">
+      <c r="E58" s="4" t="n">
         <v>79.99</v>
       </c>
-      <c r="F58" s="3" t="n">
+      <c r="F58" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G58" s="1" t="n">
@@ -2023,22 +2140,22 @@
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="3" t="s">
+      <c r="A59" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="B59" s="4" t="n">
+      <c r="B59" s="5" t="n">
         <v>45320</v>
       </c>
-      <c r="C59" s="3" t="s">
+      <c r="C59" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D59" s="4" t="n">
+      <c r="D59" s="5" t="n">
         <v>45322</v>
       </c>
-      <c r="E59" s="3" t="n">
+      <c r="E59" s="4" t="n">
         <v>49.99</v>
       </c>
-      <c r="F59" s="3" t="n">
+      <c r="F59" s="4" t="n">
         <v>3</v>
       </c>
       <c r="G59" s="1" t="n">
@@ -2047,22 +2164,22 @@
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="3" t="s">
+      <c r="A60" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="B60" s="4" t="n">
+      <c r="B60" s="5" t="n">
         <v>45321</v>
       </c>
-      <c r="C60" s="3" t="s">
+      <c r="C60" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D60" s="4" t="n">
+      <c r="D60" s="5" t="n">
         <v>45322</v>
       </c>
-      <c r="E60" s="3" t="n">
+      <c r="E60" s="4" t="n">
         <v>129.99</v>
       </c>
-      <c r="F60" s="3" t="n">
+      <c r="F60" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G60" s="1" t="n">
@@ -2071,22 +2188,22 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="3" t="s">
+      <c r="A61" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="B61" s="4" t="n">
+      <c r="B61" s="5" t="n">
         <v>45321</v>
       </c>
-      <c r="C61" s="3" t="s">
+      <c r="C61" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D61" s="4" t="n">
+      <c r="D61" s="5" t="n">
         <v>45323</v>
       </c>
-      <c r="E61" s="3" t="n">
+      <c r="E61" s="4" t="n">
         <v>19.99</v>
       </c>
-      <c r="F61" s="3" t="n">
+      <c r="F61" s="4" t="n">
         <v>4</v>
       </c>
       <c r="G61" s="1" t="n">
@@ -2095,22 +2212,22 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="3" t="s">
+      <c r="A62" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="B62" s="4" t="n">
+      <c r="B62" s="5" t="n">
         <v>45322</v>
       </c>
-      <c r="C62" s="3" t="s">
+      <c r="C62" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="D62" s="4" t="n">
+      <c r="D62" s="5" t="n">
         <v>45324</v>
       </c>
-      <c r="E62" s="3" t="n">
+      <c r="E62" s="4" t="n">
         <v>149.99</v>
       </c>
-      <c r="F62" s="3" t="n">
+      <c r="F62" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G62" s="1" t="n">
@@ -2119,22 +2236,22 @@
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="3" t="s">
+      <c r="A63" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="B63" s="4" t="n">
+      <c r="B63" s="5" t="n">
         <v>45322</v>
       </c>
-      <c r="C63" s="3" t="s">
+      <c r="C63" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D63" s="4" t="n">
+      <c r="D63" s="5" t="n">
         <v>45326</v>
       </c>
-      <c r="E63" s="3" t="n">
+      <c r="E63" s="4" t="n">
         <v>69.99</v>
       </c>
-      <c r="F63" s="3" t="n">
+      <c r="F63" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G63" s="1" t="n">
@@ -2143,22 +2260,22 @@
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="3" t="s">
+      <c r="A64" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="B64" s="4" t="n">
+      <c r="B64" s="5" t="n">
         <v>45323</v>
       </c>
-      <c r="C64" s="3" t="s">
+      <c r="C64" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="D64" s="4" t="n">
+      <c r="D64" s="5" t="n">
         <v>45324</v>
       </c>
-      <c r="E64" s="3" t="n">
+      <c r="E64" s="4" t="n">
         <v>39.99</v>
       </c>
-      <c r="F64" s="3" t="n">
+      <c r="F64" s="4" t="n">
         <v>3</v>
       </c>
       <c r="G64" s="1" t="n">
@@ -2167,22 +2284,22 @@
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="3" t="s">
+      <c r="A65" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="B65" s="4" t="n">
+      <c r="B65" s="5" t="n">
         <v>45323</v>
       </c>
-      <c r="C65" s="3" t="s">
+      <c r="C65" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D65" s="4" t="n">
+      <c r="D65" s="5" t="n">
         <v>45327</v>
       </c>
-      <c r="E65" s="3" t="n">
+      <c r="E65" s="4" t="n">
         <v>199.99</v>
       </c>
-      <c r="F65" s="3" t="n">
+      <c r="F65" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G65" s="1" t="n">
@@ -2191,22 +2308,22 @@
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="3" t="s">
+      <c r="A66" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="B66" s="4" t="n">
+      <c r="B66" s="5" t="n">
         <v>45323</v>
       </c>
-      <c r="C66" s="3" t="s">
+      <c r="C66" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="D66" s="4" t="n">
+      <c r="D66" s="5" t="n">
         <v>45325</v>
       </c>
-      <c r="E66" s="3" t="n">
+      <c r="E66" s="4" t="n">
         <v>29.99</v>
       </c>
-      <c r="F66" s="3" t="n">
+      <c r="F66" s="4" t="n">
         <v>5</v>
       </c>
       <c r="G66" s="1" t="n">
@@ -2215,22 +2332,22 @@
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="3" t="s">
+      <c r="A67" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="B67" s="4" t="n">
+      <c r="B67" s="5" t="n">
         <v>45324</v>
       </c>
-      <c r="C67" s="3" t="s">
+      <c r="C67" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="D67" s="4" t="n">
+      <c r="D67" s="5" t="n">
         <v>45328</v>
       </c>
-      <c r="E67" s="3" t="n">
+      <c r="E67" s="4" t="n">
         <v>79.99</v>
       </c>
-      <c r="F67" s="3" t="n">
+      <c r="F67" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G67" s="1" t="n">
@@ -2239,22 +2356,22 @@
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="3" t="s">
+      <c r="A68" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="B68" s="4" t="n">
+      <c r="B68" s="5" t="n">
         <v>45325</v>
       </c>
-      <c r="C68" s="3" t="s">
+      <c r="C68" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="D68" s="4" t="n">
+      <c r="D68" s="5" t="n">
         <v>45328</v>
       </c>
-      <c r="E68" s="3" t="n">
+      <c r="E68" s="4" t="n">
         <v>49.99</v>
       </c>
-      <c r="F68" s="3" t="n">
+      <c r="F68" s="4" t="n">
         <v>3</v>
       </c>
       <c r="G68" s="1" t="n">
@@ -2263,22 +2380,22 @@
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="3" t="s">
+      <c r="A69" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B69" s="4" t="n">
+      <c r="B69" s="5" t="n">
         <v>45326</v>
       </c>
-      <c r="C69" s="3" t="s">
+      <c r="C69" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D69" s="4" t="n">
+      <c r="D69" s="5" t="n">
         <v>45327</v>
       </c>
-      <c r="E69" s="3" t="n">
+      <c r="E69" s="4" t="n">
         <v>129.99</v>
       </c>
-      <c r="F69" s="3" t="n">
+      <c r="F69" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G69" s="1" t="n">
@@ -2287,22 +2404,22 @@
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="3" t="s">
+      <c r="A70" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="B70" s="4" t="n">
+      <c r="B70" s="5" t="n">
         <v>45326</v>
       </c>
-      <c r="C70" s="3" t="s">
+      <c r="C70" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D70" s="4" t="n">
+      <c r="D70" s="5" t="n">
         <v>45330</v>
       </c>
-      <c r="E70" s="3" t="n">
+      <c r="E70" s="4" t="n">
         <v>19.99</v>
       </c>
-      <c r="F70" s="3" t="n">
+      <c r="F70" s="4" t="n">
         <v>4</v>
       </c>
       <c r="G70" s="1" t="n">
@@ -2311,22 +2428,22 @@
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="3" t="s">
+      <c r="A71" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="B71" s="4" t="n">
+      <c r="B71" s="5" t="n">
         <v>45326</v>
       </c>
-      <c r="C71" s="3" t="s">
+      <c r="C71" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="D71" s="4" t="n">
+      <c r="D71" s="5" t="n">
         <v>45329</v>
       </c>
-      <c r="E71" s="3" t="n">
+      <c r="E71" s="4" t="n">
         <v>149.99</v>
       </c>
-      <c r="F71" s="3" t="n">
+      <c r="F71" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G71" s="1" t="n">
@@ -2335,10 +2452,10 @@
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B72" s="5"/>
+      <c r="B72" s="6"/>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B73" s="5"/>
+      <c r="B73" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2349,4 +2466,279 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B32"/>
+  <sheetFormatPr defaultColWidth="10.4921875" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>987</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>987</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>987</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>597</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>